<commit_message>
feat: complete Phase 5 Topwear vision extraction
</commit_message>
<xml_diff>
--- a/config/attribute_registry.xlsx
+++ b/config/attribute_registry.xlsx
@@ -8541,7 +8541,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FREE_TEXT</t>
+          <t>ENUM</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -10405,7 +10405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10424,6 +10424,36 @@
           <t>value_1</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value_2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>value_3</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>value_4</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>value_5</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>value_6</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>value_7</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -10625,7 +10655,42 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FREE_TEXT</t>
+          <t>ENUM</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Grey</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Brown</t>
         </is>
       </c>
     </row>
@@ -11430,7 +11495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11458,6 +11523,806 @@
         <is>
           <t>applicable</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>attributes__brand</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>attributes__product_type</t>
+        </is>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>attributes__model</t>
+        </is>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>attributes__color</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>attributes__size</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>attributes__material</t>
+        </is>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>attributes__fabric</t>
+        </is>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>attributes__fabric_care</t>
+        </is>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>attributes__care_instructions</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>attributes__fit</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>attributes__fit_type</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>attributes__pattern</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>attributes__pattern_type</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>attributes__design</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>attributes__neckline</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>attributes__cuff_type</t>
+        </is>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>attributes__sleeve_length</t>
+        </is>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>attributes__closure</t>
+        </is>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>attributes__fastening_type</t>
+        </is>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>attributes__comfort_level</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>attributes__finish</t>
+        </is>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>attributes__gender</t>
+        </is>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>attributes__age_group</t>
+        </is>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>attributes__season</t>
+        </is>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>attributes__occasion</t>
+        </is>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>attributes__occasion_type</t>
+        </is>
+      </c>
+      <c r="E27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>attributes__package_contents</t>
+        </is>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>attributes__in_the_box</t>
+        </is>
+      </c>
+      <c r="E29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>attributes__country_of_origin</t>
+        </is>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>attributes__weight</t>
+        </is>
+      </c>
+      <c r="E31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>attributes__product_dimensions</t>
+        </is>
+      </c>
+      <c r="E32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>topwear</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Topwear</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>topwear_mvp</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>attributes__other_information</t>
+        </is>
+      </c>
+      <c r="E33" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>